<commit_message>
adding vertical support process
</commit_message>
<xml_diff>
--- a/mock/input.xlsx
+++ b/mock/input.xlsx
@@ -5,12 +5,15 @@
   <sheets>
     <sheet state="visible" name="specs" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="updates" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="oneToMany" sheetId="3" r:id="rId6"/>
+    <sheet state="visible" name="explode" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="schema" sheetId="5" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="DSNHEJ4MnbttL070UEEwYlKSVaeH6Je3huQwIcDXGn4="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="Kgj4/vzLRQjenZlbhETpKJgQqdmdb4hXiaUalNDO9JQ="/>
     </ext>
   </extLst>
 </workbook>
@@ -36,14 +39,14 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgQZsmnraVQ+gxlIEFzNjN9aisgUQ=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miv/0lytWTAkL1f4y65tH/v8Oh4VQ=="/>
     </ext>
   </extLst>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="957" uniqueCount="346">
   <si>
     <t>Packages</t>
   </si>
@@ -2304,6 +2307,105 @@
   <si>
     <t>ADDED DISCLAIMER #237</t>
   </si>
+  <si>
+    <t>Componente</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>Versión</t>
+  </si>
+  <si>
+    <t>Servicio Asociado</t>
+  </si>
+  <si>
+    <t>Base de Datos</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>AuthService</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>v1.2</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>UserService</t>
+  </si>
+  <si>
+    <t>v1.4</t>
+  </si>
+  <si>
+    <t>OrderService</t>
+  </si>
+  <si>
+    <t>v2.0</t>
+  </si>
+  <si>
+    <t>PaymentService</t>
+  </si>
+  <si>
+    <t>v1.8</t>
+  </si>
+  <si>
+    <t>NotificationService</t>
+  </si>
+  <si>
+    <t>v1.1</t>
+  </si>
+  <si>
+    <t>Keys</t>
+  </si>
+  <si>
+    <t>a|b|c</t>
+  </si>
+  <si>
+    <t>d|e|f</t>
+  </si>
+  <si>
+    <t>h|i</t>
+  </si>
+  <si>
+    <t>z</t>
+  </si>
+  <si>
+    <t>x|y</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Attribute Name</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>UsersDB</t>
+  </si>
+  <si>
+    <t>Gateway</t>
+  </si>
+  <si>
+    <t>Stripe</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
 </sst>
 </file>
 
@@ -2314,7 +2416,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -2449,6 +2551,12 @@
       <sz val="12.0"/>
       <color rgb="FFFFFF00"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -3002,7 +3110,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="178">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3513,6 +3621,12 @@
     <xf borderId="54" fillId="0" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -3526,6 +3640,18 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -38002,4 +38128,355 @@
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="4" max="4" width="19.38"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="176" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1" s="176" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" s="176" t="s">
+        <v>315</v>
+      </c>
+      <c r="D1" s="176" t="s">
+        <v>316</v>
+      </c>
+      <c r="E1" s="176" t="s">
+        <v>317</v>
+      </c>
+      <c r="F1" s="176" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="59" t="s">
+        <v>319</v>
+      </c>
+      <c r="B2" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C2" s="59" t="s">
+        <v>321</v>
+      </c>
+      <c r="D2" s="59" t="s">
+        <v>322</v>
+      </c>
+      <c r="E2" s="59" t="s">
+        <v>322</v>
+      </c>
+      <c r="F2" s="59" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="59" t="s">
+        <v>323</v>
+      </c>
+      <c r="B3" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C3" s="59" t="s">
+        <v>324</v>
+      </c>
+      <c r="E3" s="59" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="s">
+        <v>325</v>
+      </c>
+      <c r="B4" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C4" s="59" t="s">
+        <v>326</v>
+      </c>
+      <c r="D4" s="59" t="s">
+        <v>322</v>
+      </c>
+      <c r="E4" s="59" t="s">
+        <v>322</v>
+      </c>
+      <c r="F4" s="59" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="59" t="s">
+        <v>327</v>
+      </c>
+      <c r="B5" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>328</v>
+      </c>
+      <c r="D5" s="59" t="s">
+        <v>322</v>
+      </c>
+      <c r="F5" s="59" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="59" t="s">
+        <v>329</v>
+      </c>
+      <c r="B6" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>330</v>
+      </c>
+      <c r="E6" s="59" t="s">
+        <v>322</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="176" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1" s="176" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" s="176" t="s">
+        <v>315</v>
+      </c>
+      <c r="D1" s="177" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="59" t="s">
+        <v>319</v>
+      </c>
+      <c r="B2" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C2" s="59" t="s">
+        <v>321</v>
+      </c>
+      <c r="D2" s="59" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="59" t="s">
+        <v>323</v>
+      </c>
+      <c r="B3" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C3" s="59" t="s">
+        <v>324</v>
+      </c>
+      <c r="D3" s="59" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="s">
+        <v>325</v>
+      </c>
+      <c r="B4" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C4" s="59" t="s">
+        <v>326</v>
+      </c>
+      <c r="D4" s="59" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="59" t="s">
+        <v>327</v>
+      </c>
+      <c r="B5" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>328</v>
+      </c>
+      <c r="D5" s="59" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="59" t="s">
+        <v>329</v>
+      </c>
+      <c r="B6" s="59" t="s">
+        <v>320</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>330</v>
+      </c>
+      <c r="D6" s="59" t="s">
+        <v>336</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="21.75"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="176" t="s">
+        <v>337</v>
+      </c>
+      <c r="B1" s="176" t="s">
+        <v>338</v>
+      </c>
+      <c r="C1" s="176" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="59" t="s">
+        <v>319</v>
+      </c>
+      <c r="B2" s="59" t="s">
+        <v>314</v>
+      </c>
+      <c r="C2" s="59" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="59" t="s">
+        <v>319</v>
+      </c>
+      <c r="B3" s="59" t="s">
+        <v>315</v>
+      </c>
+      <c r="C3" s="59" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="59" t="s">
+        <v>323</v>
+      </c>
+      <c r="B5" s="59" t="s">
+        <v>314</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="59" t="s">
+        <v>323</v>
+      </c>
+      <c r="B6" s="59" t="s">
+        <v>315</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="59" t="s">
+        <v>323</v>
+      </c>
+      <c r="B7" s="59" t="s">
+        <v>340</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="59"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="59"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="59" t="s">
+        <v>327</v>
+      </c>
+      <c r="B9" s="59" t="s">
+        <v>314</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="59" t="s">
+        <v>327</v>
+      </c>
+      <c r="B10" s="59" t="s">
+        <v>315</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="59" t="s">
+        <v>327</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>342</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="59" t="s">
+        <v>327</v>
+      </c>
+      <c r="B12" s="59" t="s">
+        <v>344</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>345</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updating to add support to required fields
</commit_message>
<xml_diff>
--- a/mock/input.xlsx
+++ b/mock/input.xlsx
@@ -13,7 +13,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="Kgj4/vzLRQjenZlbhETpKJgQqdmdb4hXiaUalNDO9JQ="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="VLhpHpUl6wV/vEJuQyDn6vzR2GPvwL9vP5SefqxZX7A="/>
     </ext>
   </extLst>
 </workbook>
@@ -39,14 +39,14 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miv/0lytWTAkL1f4y65tH/v8Oh4VQ=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhpc4WtxcSRdbC3e/bbFWo6xvMa2A=="/>
     </ext>
   </extLst>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="957" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="345">
   <si>
     <t>Packages</t>
   </si>
@@ -2398,9 +2398,6 @@
     <t>Gateway</t>
   </si>
   <si>
-    <t>Stripe</t>
-  </si>
-  <si>
     <t>Currency</t>
   </si>
   <si>
@@ -38306,9 +38303,6 @@
       <c r="B4" s="59" t="s">
         <v>320</v>
       </c>
-      <c r="C4" s="59" t="s">
-        <v>326</v>
-      </c>
       <c r="D4" s="59" t="s">
         <v>334</v>
       </c>
@@ -38461,19 +38455,16 @@
       <c r="B11" s="59" t="s">
         <v>342</v>
       </c>
-      <c r="C11" s="59" t="s">
-        <v>343</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="59" t="s">
         <v>327</v>
       </c>
       <c r="B12" s="59" t="s">
+        <v>343</v>
+      </c>
+      <c r="C12" s="59" t="s">
         <v>344</v>
-      </c>
-      <c r="C12" s="59" t="s">
-        <v>345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding support ro resolver relationship
</commit_message>
<xml_diff>
--- a/mock/input.xlsx
+++ b/mock/input.xlsx
@@ -70,7 +70,7 @@
         <t xml:space="preserve">======
 ID#AAAB1_VdfyU
 Alexander Wong    (2026-03-17 15:29:52)
-Title: Engine Type: 1.5L VTEC® Turbo Inline-4
+Headline: Engine Type: 1.5L VTEC® Turbo Inline-4
 Description: The turbocharged Integra is engineered for true driving enthusiasts. With a 1.5L VTEC® Turbo engine that pumps out 200-HP* and an early and flat torque curve that offers smooth power delivery, the Integra is a powerful and agile tour de force.
 Image:  /-/media/Acura-Platform/Vehicle-Pages/INTEGRA/2025/pricing-and-specs/Specs-Cards-Powertrain/In-Line-4-Cylinder/Acura-Integra-Pricing-and-Specs-powertrain-s.jpg</t>
       </text>
@@ -89,7 +89,7 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgQcyu16xD1mmvLjK41Jg3neVlDiA=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhubDM2u3HqRvardiPDUmGzgGpoUg=="/>
     </ext>
   </extLst>
 </comments>

</xml_diff>